<commit_message>
Close pilot botanical database v1.0
</commit_message>
<xml_diff>
--- a/data/source/Fichas_especies_arboris.xlsx
+++ b/data/source/Fichas_especies_arboris.xlsx
@@ -2,26 +2,31 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Indice" sheetId="1" r:id="R2c626320aae44e2c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Peumo" sheetId="2" r:id="R1cff3282c16d41c9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Litre" sheetId="3" r:id="R07e6c9daacb2439a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bollen" sheetId="4" r:id="R705d92f6d163466d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mitique" sheetId="5" r:id="Rfc46496453864005"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Colliguay" sheetId="6" r:id="R0811c1d376ff433d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quillay" sheetId="7" r:id="R28058e8fa95d414a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fuentes" sheetId="8" r:id="Rc27bc8d7e2aa4738"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fotos" sheetId="9" r:id="Rea2a0f0c5f8041de"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Individuos" sheetId="10" r:id="R16af0812ad1e41c7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Observaciones" sheetId="11" r:id="Re9a404192bcf4b79"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Caracteres" sheetId="12" r:id="R3718eb5dfcee49e5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Estados_caracteres" sheetId="13" r:id="R2665db14512b4046"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Errores_identificacion" sheetId="14" r:id="Ra8317888440f4619"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mapa_legacy_caracteres" sheetId="15" r:id="Ra9bc53abbf98425c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LEEME" sheetId="16" r:id="R41e747811b614790"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Respuestas_observacion" sheetId="17" r:id="R7b03dfaca1b84e60"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Estados_retirados" sheetId="18" r:id="R78082f4654e545ab"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Auditoria_atomicidad" sheetId="19" r:id="Rf0adf919f2124754"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Especie_Caracter" sheetId="20" r:id="R9c0e01d9326c4231"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Indice" sheetId="1" r:id="R2c065b807abe4284"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Peumo" sheetId="2" r:id="R5d4e9f39d3af49d3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Litre" sheetId="3" r:id="R478ab38ca11842b3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bollen" sheetId="4" r:id="Rc006f84643ce49dc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mitique" sheetId="5" r:id="R8dd1ee133b5c4f38"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Colliguay" sheetId="6" r:id="R45b2f6b77e674e9a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quillay" sheetId="7" r:id="R072ffda9161f457f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fuentes" sheetId="8" r:id="R6d2ac9cc83ec47c1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fotos" sheetId="9" r:id="Ree2735739bb64e49"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Individuos" sheetId="10" r:id="Rbd964dd5c57d4e77"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Observaciones" sheetId="11" r:id="Rd9b04fc508354d21"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Caracteres" sheetId="12" r:id="R8d9d0215663042d2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Estados_caracteres" sheetId="13" r:id="Rf35c563723ab4de2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Errores_identificacion" sheetId="14" r:id="R9893c51c1c354089"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mapa_legacy_caracteres" sheetId="15" r:id="Rb4de2cafbcd340a5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LEEME" sheetId="16" r:id="Rf2d8818573804939"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Respuestas_observacion" sheetId="17" r:id="R1e1ef9036a8b4841"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Estados_retirados" sheetId="18" r:id="Rb6560d1499774438"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Auditoria_atomicidad" sheetId="19" r:id="R5da096460fd848f1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Especie_Caracter" sheetId="20" r:id="Rfc189e8c63bc4521"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Taxonomia" sheetId="21" r:id="R231f5abe42a44951"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Contexto_especie" sheetId="22" r:id="R2c5b5ed4a7594bad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Diagnostico_piloto" sheetId="23" r:id="R84ab5eb704234b8d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Observabilidad_piloto" sheetId="24" r:id="R0a581e7ae09f43dc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Control_version" sheetId="25" r:id="R4f17244fb6214b20"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -84,7 +89,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="37">
+  <x:fills count="39">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -266,6 +271,16 @@
         <x:fgColor rgb="FF355E3B"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF587A5B"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFDCE8DC"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="18">
     <x:border/>
@@ -290,7 +305,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="237">
+  <x:cellXfs count="246">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -830,6 +845,29 @@
     <x:xf numFmtId="0" fontId="2" fillId="36" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="37" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="37" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="37" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="37" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="37" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="38" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="38" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="38" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -1139,6 +1177,11 @@
       <x:c r="G1" s="5"/>
       <x:c r="H1" s="5"/>
     </x:row>
+    <x:row r="2">
+      <x:c r="F2" t="str">
+        <x:v>Ficha botánica v1.0</x:v>
+      </x:c>
+    </x:row>
     <x:row r="3">
       <x:c r="A3" s="13" t="str">
         <x:v>ID</x:v>
@@ -1156,7 +1199,7 @@
         <x:v>Hábito</x:v>
       </x:c>
       <x:c r="F3" s="13" t="str">
-        <x:v>Estado ficha</x:v>
+        <x:v>Ficha botánica v1.0</x:v>
       </x:c>
       <x:c r="G3" s="173" t="str">
         <x:v>Fotos registradas</x:v>
@@ -1188,7 +1231,7 @@
         <x:v>Árbol</x:v>
       </x:c>
       <x:c r="F4" s="28" t="str">
-        <x:v>Ficha avanzada</x:v>
+        <x:v>Ficha botánica v1.0</x:v>
       </x:c>
       <x:c r="G4" s="171" t="n">
         <x:f>COUNTIF(Fotos!$B$2:$B$46,A4)</x:f>
@@ -1223,7 +1266,7 @@
         <x:v>Árbol</x:v>
       </x:c>
       <x:c r="F5" s="31" t="str">
-        <x:v>Ficha avanzada</x:v>
+        <x:v>Ficha botánica v1.0</x:v>
       </x:c>
       <x:c r="G5" s="171" t="n">
         <x:f>COUNTIF(Fotos!$B$2:$B$46,A5)</x:f>
@@ -1258,7 +1301,7 @@
         <x:v>Árbol/arbusto</x:v>
       </x:c>
       <x:c r="F6" s="31" t="str">
-        <x:v>Ficha avanzada</x:v>
+        <x:v>Ficha botánica v1.0</x:v>
       </x:c>
       <x:c r="G6" s="171" t="n">
         <x:f>COUNTIF(Fotos!$B$2:$B$46,A6)</x:f>
@@ -1293,7 +1336,7 @@
         <x:v>Arbusto</x:v>
       </x:c>
       <x:c r="F7" s="31" t="str">
-        <x:v>Ficha avanzada</x:v>
+        <x:v>Ficha botánica v1.0</x:v>
       </x:c>
       <x:c r="G7" s="171" t="n">
         <x:f>COUNTIF(Fotos!$B$2:$B$46,A7)</x:f>
@@ -1984,7 +2027,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc6ec88b4627f453f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R87734d0a4e2942c6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2591,7 +2634,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8d0a82aed0f04312"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3640d2bf3d204ba4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2614,37 +2657,37 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="192" t="str">
+      <x:c r="A1" s="238" t="str">
         <x:v>ID carácter</x:v>
       </x:c>
-      <x:c r="B1" s="192" t="str">
+      <x:c r="B1" s="238" t="str">
         <x:v>Órgano / estructura</x:v>
       </x:c>
-      <x:c r="C1" s="192" t="str">
+      <x:c r="C1" s="238" t="str">
         <x:v>Nombre normalizado</x:v>
       </x:c>
-      <x:c r="D1" s="192" t="str">
+      <x:c r="D1" s="238" t="str">
         <x:v>Tipo de dato</x:v>
       </x:c>
-      <x:c r="E1" s="192" t="str">
+      <x:c r="E1" s="238" t="str">
         <x:v>Estados registrados en el piloto</x:v>
       </x:c>
-      <x:c r="F1" s="192" t="str">
-        <x:v>Detectabilidad registrada</x:v>
-      </x:c>
-      <x:c r="G1" s="192" t="str">
+      <x:c r="F1" s="238" t="str">
+        <x:v>Detectabilidad en imagen (resumen piloto)</x:v>
+      </x:c>
+      <x:c r="G1" s="238" t="str">
         <x:v>Seguridad / interacción registrada</x:v>
       </x:c>
-      <x:c r="H1" s="192" t="str">
+      <x:c r="H1" s="238" t="str">
         <x:v>Especies del piloto</x:v>
       </x:c>
-      <x:c r="I1" s="192" t="str">
+      <x:c r="I1" s="238" t="str">
         <x:v>Notas</x:v>
       </x:c>
-      <x:c r="J1" s="200" t="str">
+      <x:c r="J1" s="238" t="str">
         <x:v>Estados controlados en</x:v>
       </x:c>
-      <x:c r="K1" s="200" t="str">
+      <x:c r="K1" s="238" t="str">
         <x:v>Regla de almacenamiento</x:v>
       </x:c>
     </x:row>
@@ -2730,7 +2773,7 @@
         <x:v>categórico</x:v>
       </x:c>
       <x:c r="E4" s="85" t="str">
-        <x:v>entero | ondulado | serrado | aserrado | discretamente dentado</x:v>
+        <x:v>entero | serrado | aserrado | discretamente dentado</x:v>
       </x:c>
       <x:c r="F4" s="85" t="str">
         <x:v>Sí</x:v>
@@ -2741,7 +2784,9 @@
       <x:c r="H4" s="85" t="str">
         <x:v>Peumo | Litre | Bollén | Mitique | Colliguay | Quillay</x:v>
       </x:c>
-      <x:c r="I4" s="85" t="str"/>
+      <x:c r="I4" s="85" t="str">
+        <x:v>Describe dentición del margen. 'Ondulado' se separa en CAR-037 porque una hoja puede ser simultáneamente entera y ondulada.</x:v>
+      </x:c>
       <x:c r="J4" t="str">
         <x:v>Estados_caracteres</x:v>
       </x:c>
@@ -3937,6 +3982,41 @@
         <x:v>Estados_caracteres</x:v>
       </x:c>
       <x:c r="K41" s="85" t="str">
+        <x:v>Uno o más ID/estados normalizados; nunca texto libre</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42">
+      <x:c r="A42" t="str">
+        <x:v>CAR-037</x:v>
+      </x:c>
+      <x:c r="B42" t="str">
+        <x:v>Hoja</x:v>
+      </x:c>
+      <x:c r="C42" t="str">
+        <x:v>Ondulación del margen</x:v>
+      </x:c>
+      <x:c r="D42" t="str">
+        <x:v>categórico</x:v>
+      </x:c>
+      <x:c r="E42" t="str">
+        <x:v>ondulado</x:v>
+      </x:c>
+      <x:c r="F42" t="str">
+        <x:v>Sí</x:v>
+      </x:c>
+      <x:c r="G42" t="str">
+        <x:v>seguro | precaucion</x:v>
+      </x:c>
+      <x:c r="H42" t="str">
+        <x:v>Peumo | Litre</x:v>
+      </x:c>
+      <x:c r="I42" t="str">
+        <x:v>Separado de CAR-003: la ondulación no es una categoría de dentición.</x:v>
+      </x:c>
+      <x:c r="J42" t="str">
+        <x:v>Estados_caracteres</x:v>
+      </x:c>
+      <x:c r="K42" t="str">
         <x:v>Uno o más ID/estados normalizados; nunca texto libre</x:v>
       </x:c>
     </x:row>
@@ -5214,6 +5294,24 @@
         <x:v>flor femenina en la base del amento</x:v>
       </x:c>
       <x:c r="F75" s="85"/>
+    </x:row>
+    <x:row r="76">
+      <x:c r="A76" t="str">
+        <x:v>EST-037-01</x:v>
+      </x:c>
+      <x:c r="B76" t="str">
+        <x:v>CAR-037</x:v>
+      </x:c>
+      <x:c r="C76" t="str">
+        <x:v>ondulado</x:v>
+      </x:c>
+      <x:c r="D76" t="str">
+        <x:v>Ondulado</x:v>
+      </x:c>
+      <x:c r="E76"/>
+      <x:c r="F76" t="str">
+        <x:v>Estado transferido desde EST-003-02 tras separar ondulación de dentición.</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -5766,10 +5864,10 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="212" t="str">
+      <x:c r="A1" s="214" t="str">
         <x:v>Árboris — Base editorial canónica del piloto</x:v>
       </x:c>
-      <x:c r="B1" s="212" t="str"/>
+      <x:c r="B1" s="214" t="str"/>
       <x:c r="C1" s="212" t="str"/>
       <x:c r="D1" s="212" t="str"/>
     </x:row>
@@ -5854,10 +5952,10 @@
       <x:c r="D9" s="85" t="str"/>
     </x:row>
     <x:row r="10">
-      <x:c r="A10" s="227" t="str">
+      <x:c r="A10" s="195" t="str">
         <x:v>Regla de estados biológicos</x:v>
       </x:c>
-      <x:c r="B10" s="227" t="str"/>
+      <x:c r="B10" s="195" t="str"/>
       <x:c r="C10" s="227" t="str"/>
       <x:c r="D10" s="227" t="str"/>
     </x:row>
@@ -5892,10 +5990,10 @@
       <x:c r="D13" s="85" t="str"/>
     </x:row>
     <x:row r="14">
-      <x:c r="A14" s="235" t="str">
+      <x:c r="A14" s="195" t="str">
         <x:v>Regla de atomicidad</x:v>
       </x:c>
-      <x:c r="B14" s="235" t="str"/>
+      <x:c r="B14" s="195" t="str"/>
       <x:c r="C14" s="235" t="str"/>
       <x:c r="D14" s="235" t="str"/>
     </x:row>
@@ -5938,6 +6036,62 @@
       </x:c>
       <x:c r="C18" s="85" t="str"/>
       <x:c r="D18" s="85" t="str"/>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="244" t="str">
+        <x:v>Cierre v1.0</x:v>
+      </x:c>
+      <x:c r="B19" s="85" t="str">
+        <x:v>La base botánica queda cerrada editorialmente para las seis especies del piloto. Cualquier ampliación taxonómica o incorporación de nuevas especies debe abrir una nueva versión.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="244" t="str">
+        <x:v>Poder diagnóstico</x:v>
+      </x:c>
+      <x:c r="B20" s="85" t="str">
+        <x:v>Las columnas de poder diagnóstico se interpretan exclusivamente dentro del piloto de seis especies. El valor depende del conjunto candidato y puede cambiar dinámicamente durante una identificación.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="244" t="str">
+        <x:v>Confianza especie–carácter</x:v>
+      </x:c>
+      <x:c r="B21" s="85" t="str">
+        <x:v>La columna de confianza indica respaldo de la asignación botánica especie–carácter/estado. No equivale a la confianza de una identificación de usuario.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="244" t="str">
+        <x:v>Detectabilidad</x:v>
+      </x:c>
+      <x:c r="B22" s="85" t="str">
+        <x:v>La detectabilidad registrada en las fichas resume el piloto. La hoja Observabilidad_piloto separa la utilidad visual/fotográfica de las restricciones de interacción.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="244" t="str">
+        <x:v>Margen foliar</x:v>
+      </x:c>
+      <x:c r="B23" s="85" t="str">
+        <x:v>CAR-003 representa dentición. La ondulación se registra por separado en CAR-037; EST-003-02 fue retirado y reemplazado por EST-037-01.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="244" t="str">
+        <x:v>Taxonomía</x:v>
+      </x:c>
+      <x:c r="B24" s="85" t="str">
+        <x:v>La hoja Taxonomia incorpora autoría, estado aceptado y LSID POWO/IPNI como backbone complementario. F-001 continúa siendo la autoridad chilena principal del proyecto.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="244" t="str">
+        <x:v>Validación pendiente</x:v>
+      </x:c>
+      <x:c r="B25" s="85" t="str">
+        <x:v>El cierre editorial no equivale a validación del motor de identificación. Falta probar la clave y la observabilidad contra las 45 fotografías de referencia.</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -6481,6 +6635,26 @@
       </x:c>
       <x:c r="F22" s="85" t="str">
         <x:v>CAR-012 fue atomizado en CAR-031 a CAR-036; conservar solo para trazabilidad.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" t="str">
+        <x:v>EST-003-02</x:v>
+      </x:c>
+      <x:c r="B23" t="str">
+        <x:v>CAR-003</x:v>
+      </x:c>
+      <x:c r="C23" t="str">
+        <x:v>ondulado</x:v>
+      </x:c>
+      <x:c r="D23" t="str">
+        <x:v>Ondulado</x:v>
+      </x:c>
+      <x:c r="E23" t="str">
+        <x:v>retirado</x:v>
+      </x:c>
+      <x:c r="F23" t="str">
+        <x:v>La ondulación no es una categoría de dentición. Se reemplaza por CAR-037 / EST-037-01.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -6916,6 +7090,32 @@
       </x:c>
       <x:c r="H16" s="85" t="str">
         <x:v>No se interpreta la discrepancia como variación biológica.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" t="str">
+        <x:v>Margen entero|ondulado</x:v>
+      </x:c>
+      <x:c r="B17" t="str">
+        <x:v>Mezclaba dentición con ondulación del borde</x:v>
+      </x:c>
+      <x:c r="C17" t="str">
+        <x:v>Separar</x:v>
+      </x:c>
+      <x:c r="D17" t="str">
+        <x:v>CAR-003=dentición; CAR-037=ondulación</x:v>
+      </x:c>
+      <x:c r="E17" t="str">
+        <x:v>Peumo, Litre</x:v>
+      </x:c>
+      <x:c r="F17" t="str">
+        <x:v>CAR-037 / EST-037-01</x:v>
+      </x:c>
+      <x:c r="G17" t="str">
+        <x:v>implementado</x:v>
+      </x:c>
+      <x:c r="H17" t="str">
+        <x:v>Una hoja puede ser entera y ondulada simultáneamente; se evita tratarlos como estados excluyentes.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -7041,11 +7241,33 @@
         <x:v>Estado de ficha</x:v>
       </x:c>
       <x:c r="E8" t="str">
-        <x:v>Ficha avanzada</x:v>
+        <x:v>Ficha botánica v1.0</x:v>
       </x:c>
       <x:c r="F8" t="str"/>
       <x:c r="G8" t="str"/>
       <x:c r="H8" t="str"/>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="245" t="str">
+        <x:v>Autoría taxonómica</x:v>
+      </x:c>
+      <x:c r="B9" s="85" t="str">
+        <x:v>(Molina) Looser</x:v>
+      </x:c>
+      <x:c r="C9" s="85"/>
+      <x:c r="D9" s="245" t="str">
+        <x:v>POWO/IPNI LSID</x:v>
+      </x:c>
+      <x:c r="E9" s="85" t="str">
+        <x:v>urn:lsid:ipni.org:names:1125917-2</x:v>
+      </x:c>
+      <x:c r="F9" s="85"/>
+      <x:c r="G9" s="245" t="str">
+        <x:v>Fuente</x:v>
+      </x:c>
+      <x:c r="H9" s="85" t="str">
+        <x:v>F-020</x:v>
+      </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="66" t="str">
@@ -7104,34 +7326,34 @@
       <x:c r="H15" s="66"/>
     </x:row>
     <x:row r="16">
-      <x:c r="A16" s="78" t="str">
+      <x:c r="A16" s="238" t="str">
         <x:v>Carácter</x:v>
       </x:c>
-      <x:c r="B16" s="78" t="str">
+      <x:c r="B16" s="238" t="str">
         <x:v>Estado esperado</x:v>
       </x:c>
-      <x:c r="C16" s="78" t="str">
+      <x:c r="C16" s="238" t="str">
         <x:v>Variabilidad</x:v>
       </x:c>
-      <x:c r="D16" s="78" t="str">
-        <x:v>Detectable en imagen</x:v>
-      </x:c>
-      <x:c r="E16" s="78" t="str">
-        <x:v>Poder diagnóstico</x:v>
-      </x:c>
-      <x:c r="F16" s="78" t="str">
+      <x:c r="D16" s="238" t="str">
+        <x:v>Detectabilidad en imagen (piloto)</x:v>
+      </x:c>
+      <x:c r="E16" s="238" t="str">
+        <x:v>Poder diagnóstico (piloto)</x:v>
+      </x:c>
+      <x:c r="F16" s="238" t="str">
         <x:v>Seguridad</x:v>
       </x:c>
-      <x:c r="G16" s="78" t="str">
-        <x:v>Confianza</x:v>
-      </x:c>
-      <x:c r="H16" s="78" t="str">
+      <x:c r="G16" s="238" t="str">
+        <x:v>Confianza asignación especie–carácter</x:v>
+      </x:c>
+      <x:c r="H16" s="238" t="str">
         <x:v>Fuente</x:v>
       </x:c>
-      <x:c r="I16" s="192" t="str">
+      <x:c r="I16" s="238" t="str">
         <x:v>ID carácter</x:v>
       </x:c>
-      <x:c r="J16" s="192" t="str">
+      <x:c r="J16" s="238" t="str">
         <x:v>Estado normalización</x:v>
       </x:c>
     </x:row>
@@ -7204,7 +7426,7 @@
         <x:v>Margen foliar</x:v>
       </x:c>
       <x:c r="B19" s="94" t="str">
-        <x:v>entero|ondulado</x:v>
+        <x:v>entero</x:v>
       </x:c>
       <x:c r="C19" s="94" t="str">
         <x:v>media</x:v>
@@ -7552,8 +7774,36 @@
       </x:c>
     </x:row>
     <x:row r="30">
-      <x:c r="I30" s="85"/>
-      <x:c r="J30" s="85"/>
+      <x:c r="A30" s="85" t="str">
+        <x:v>Ondulación del margen</x:v>
+      </x:c>
+      <x:c r="B30" s="85" t="str">
+        <x:v>ondulado</x:v>
+      </x:c>
+      <x:c r="C30" s="85" t="str">
+        <x:v>media</x:v>
+      </x:c>
+      <x:c r="D30" s="85" t="str">
+        <x:v>Sí</x:v>
+      </x:c>
+      <x:c r="E30" s="85" t="str">
+        <x:v>medio</x:v>
+      </x:c>
+      <x:c r="F30" s="85" t="str">
+        <x:v>seguro</x:v>
+      </x:c>
+      <x:c r="G30" s="85" t="str">
+        <x:v>alta</x:v>
+      </x:c>
+      <x:c r="H30" s="85" t="str">
+        <x:v>F-002</x:v>
+      </x:c>
+      <x:c r="I30" s="85" t="str">
+        <x:v>CAR-037</x:v>
+      </x:c>
+      <x:c r="J30" s="85" t="str">
+        <x:v>normalizado</x:v>
+      </x:c>
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="66" t="str">
@@ -7860,43 +8110,43 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="236" t="str">
+      <x:c r="A1" s="238" t="str">
         <x:v>Especie ID</x:v>
       </x:c>
-      <x:c r="B1" s="236" t="str">
+      <x:c r="B1" s="238" t="str">
         <x:v>Nombre común</x:v>
       </x:c>
-      <x:c r="C1" s="236" t="str">
+      <x:c r="C1" s="238" t="str">
         <x:v>ID carácter</x:v>
       </x:c>
-      <x:c r="D1" s="236" t="str">
+      <x:c r="D1" s="238" t="str">
         <x:v>Carácter</x:v>
       </x:c>
-      <x:c r="E1" s="236" t="str">
+      <x:c r="E1" s="238" t="str">
         <x:v>ID estado</x:v>
       </x:c>
-      <x:c r="F1" s="236" t="str">
+      <x:c r="F1" s="238" t="str">
         <x:v>Estado</x:v>
       </x:c>
-      <x:c r="G1" s="236" t="str">
+      <x:c r="G1" s="238" t="str">
         <x:v>Variabilidad</x:v>
       </x:c>
-      <x:c r="H1" s="236" t="str">
-        <x:v>Detectable en imagen</x:v>
-      </x:c>
-      <x:c r="I1" s="236" t="str">
-        <x:v>Poder diagnóstico</x:v>
-      </x:c>
-      <x:c r="J1" s="236" t="str">
+      <x:c r="H1" s="238" t="str">
+        <x:v>Detectabilidad en imagen (piloto)</x:v>
+      </x:c>
+      <x:c r="I1" s="238" t="str">
+        <x:v>Poder diagnóstico (piloto)</x:v>
+      </x:c>
+      <x:c r="J1" s="238" t="str">
         <x:v>Seguridad</x:v>
       </x:c>
-      <x:c r="K1" s="236" t="str">
-        <x:v>Confianza</x:v>
-      </x:c>
-      <x:c r="L1" s="236" t="str">
+      <x:c r="K1" s="238" t="str">
+        <x:v>Confianza asignación especie–carácter</x:v>
+      </x:c>
+      <x:c r="L1" s="238" t="str">
         <x:v>Fuente</x:v>
       </x:c>
-      <x:c r="M1" s="236" t="str">
+      <x:c r="M1" s="238" t="str">
         <x:v>Estado normalización</x:v>
       </x:c>
     </x:row>
@@ -8113,13 +8363,13 @@
         <x:v>Peumo</x:v>
       </x:c>
       <x:c r="C7" s="85" t="str">
-        <x:v>CAR-003</x:v>
+        <x:v>CAR-037</x:v>
       </x:c>
       <x:c r="D7" s="85" t="str">
-        <x:v>Margen foliar</x:v>
+        <x:v>Ondulación del margen</x:v>
       </x:c>
       <x:c r="E7" s="85" t="str">
-        <x:v>EST-003-02</x:v>
+        <x:v>EST-037-01</x:v>
       </x:c>
       <x:c r="F7" s="85" t="str">
         <x:v>ondulado</x:v>
@@ -8851,13 +9101,13 @@
         <x:v>Litre</x:v>
       </x:c>
       <x:c r="C25" s="85" t="str">
-        <x:v>CAR-003</x:v>
+        <x:v>CAR-037</x:v>
       </x:c>
       <x:c r="D25" s="85" t="str">
-        <x:v>Margen foliar</x:v>
+        <x:v>Ondulación del margen</x:v>
       </x:c>
       <x:c r="E25" s="85" t="str">
-        <x:v>EST-003-02</x:v>
+        <x:v>EST-037-01</x:v>
       </x:c>
       <x:c r="F25" s="85" t="str">
         <x:v>ondulado</x:v>
@@ -12408,6 +12658,1313 @@
       </x:c>
       <x:c r="M111" s="85" t="str">
         <x:v>normalizado</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="12" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="14" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="24" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="22" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="18" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="16" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="16" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="30" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="38" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="10" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="238" t="str">
+        <x:v>Especie ID</x:v>
+      </x:c>
+      <x:c r="B1" s="238" t="str">
+        <x:v>Nombre común</x:v>
+      </x:c>
+      <x:c r="C1" s="238" t="str">
+        <x:v>Nombre aceptado</x:v>
+      </x:c>
+      <x:c r="D1" s="238" t="str">
+        <x:v>Autoría</x:v>
+      </x:c>
+      <x:c r="E1" s="238" t="str">
+        <x:v>Familia</x:v>
+      </x:c>
+      <x:c r="F1" s="238" t="str">
+        <x:v>Orden</x:v>
+      </x:c>
+      <x:c r="G1" s="238" t="str">
+        <x:v>Estado taxonómico</x:v>
+      </x:c>
+      <x:c r="H1" s="238" t="str">
+        <x:v>POWO/IPNI LSID</x:v>
+      </x:c>
+      <x:c r="I1" s="238" t="str">
+        <x:v>Rango nativo POWO</x:v>
+      </x:c>
+      <x:c r="J1" s="238" t="str">
+        <x:v>Fuente</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="85" t="str">
+        <x:v>SP-001</x:v>
+      </x:c>
+      <x:c r="B2" s="85" t="str">
+        <x:v>Peumo</x:v>
+      </x:c>
+      <x:c r="C2" s="85" t="str">
+        <x:v>Cryptocarya alba</x:v>
+      </x:c>
+      <x:c r="D2" s="85" t="str">
+        <x:v>(Molina) Looser</x:v>
+      </x:c>
+      <x:c r="E2" s="85" t="str">
+        <x:v>Lauraceae</x:v>
+      </x:c>
+      <x:c r="F2" s="85" t="str">
+        <x:v>Laurales</x:v>
+      </x:c>
+      <x:c r="G2" s="85" t="str">
+        <x:v>aceptado</x:v>
+      </x:c>
+      <x:c r="H2" s="85" t="str">
+        <x:v>urn:lsid:ipni.org:names:1125917-2</x:v>
+      </x:c>
+      <x:c r="I2" s="85" t="str">
+        <x:v>Chile Central y Chile Sur (hasta N de Los Lagos)</x:v>
+      </x:c>
+      <x:c r="J2" s="85" t="str">
+        <x:v>F-020</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="85" t="str">
+        <x:v>SP-002</x:v>
+      </x:c>
+      <x:c r="B3" s="85" t="str">
+        <x:v>Litre</x:v>
+      </x:c>
+      <x:c r="C3" s="85" t="str">
+        <x:v>Lithraea caustica</x:v>
+      </x:c>
+      <x:c r="D3" s="85" t="str">
+        <x:v>(Molina) Hook. &amp; Arn.</x:v>
+      </x:c>
+      <x:c r="E3" s="85" t="str">
+        <x:v>Anacardiaceae</x:v>
+      </x:c>
+      <x:c r="F3" s="85" t="str">
+        <x:v>Sapindales</x:v>
+      </x:c>
+      <x:c r="G3" s="85" t="str">
+        <x:v>aceptado</x:v>
+      </x:c>
+      <x:c r="H3" s="85" t="str">
+        <x:v>urn:lsid:ipni.org:names:69838-1</x:v>
+      </x:c>
+      <x:c r="I3" s="85" t="str">
+        <x:v>Chile Central</x:v>
+      </x:c>
+      <x:c r="J3" s="85" t="str">
+        <x:v>F-020</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="85" t="str">
+        <x:v>SP-003</x:v>
+      </x:c>
+      <x:c r="B4" s="85" t="str">
+        <x:v>Bollén</x:v>
+      </x:c>
+      <x:c r="C4" s="85" t="str">
+        <x:v>Kageneckia oblonga</x:v>
+      </x:c>
+      <x:c r="D4" s="85" t="str">
+        <x:v>Ruiz &amp; Pav.</x:v>
+      </x:c>
+      <x:c r="E4" s="85" t="str">
+        <x:v>Rosaceae</x:v>
+      </x:c>
+      <x:c r="F4" s="85" t="str">
+        <x:v>Rosales</x:v>
+      </x:c>
+      <x:c r="G4" s="85" t="str">
+        <x:v>aceptado</x:v>
+      </x:c>
+      <x:c r="H4" s="85" t="str">
+        <x:v>urn:lsid:ipni.org:names:725811-1</x:v>
+      </x:c>
+      <x:c r="I4" s="85" t="str">
+        <x:v>Chile Central</x:v>
+      </x:c>
+      <x:c r="J4" s="85" t="str">
+        <x:v>F-020</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="85" t="str">
+        <x:v>SP-004</x:v>
+      </x:c>
+      <x:c r="B5" s="85" t="str">
+        <x:v>Mitique</x:v>
+      </x:c>
+      <x:c r="C5" s="85" t="str">
+        <x:v>Podanthus mitiqui</x:v>
+      </x:c>
+      <x:c r="D5" s="85" t="str">
+        <x:v>Lindl.</x:v>
+      </x:c>
+      <x:c r="E5" s="85" t="str">
+        <x:v>Asteraceae</x:v>
+      </x:c>
+      <x:c r="F5" s="85" t="str">
+        <x:v>Asterales</x:v>
+      </x:c>
+      <x:c r="G5" s="85" t="str">
+        <x:v>aceptado</x:v>
+      </x:c>
+      <x:c r="H5" s="85" t="str">
+        <x:v>urn:lsid:ipni.org:names:238927-1</x:v>
+      </x:c>
+      <x:c r="I5" s="85" t="str">
+        <x:v>Norte-centro y centro de Chile</x:v>
+      </x:c>
+      <x:c r="J5" s="85" t="str">
+        <x:v>F-020</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="85" t="str">
+        <x:v>SP-005</x:v>
+      </x:c>
+      <x:c r="B6" s="85" t="str">
+        <x:v>Colliguay</x:v>
+      </x:c>
+      <x:c r="C6" s="85" t="str">
+        <x:v>Colliguaja odorifera</x:v>
+      </x:c>
+      <x:c r="D6" s="85" t="str">
+        <x:v>Molina</x:v>
+      </x:c>
+      <x:c r="E6" s="85" t="str">
+        <x:v>Euphorbiaceae</x:v>
+      </x:c>
+      <x:c r="F6" s="85" t="str">
+        <x:v>Malpighiales</x:v>
+      </x:c>
+      <x:c r="G6" s="85" t="str">
+        <x:v>aceptado</x:v>
+      </x:c>
+      <x:c r="H6" s="85" t="str">
+        <x:v>urn:lsid:ipni.org:names:341899-1</x:v>
+      </x:c>
+      <x:c r="I6" s="85" t="str">
+        <x:v>Norte y centro de Chile</x:v>
+      </x:c>
+      <x:c r="J6" s="85" t="str">
+        <x:v>F-020</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="85" t="str">
+        <x:v>SP-006</x:v>
+      </x:c>
+      <x:c r="B7" s="85" t="str">
+        <x:v>Quillay</x:v>
+      </x:c>
+      <x:c r="C7" s="85" t="str">
+        <x:v>Quillaja saponaria</x:v>
+      </x:c>
+      <x:c r="D7" s="85" t="str">
+        <x:v>Molina</x:v>
+      </x:c>
+      <x:c r="E7" s="85" t="str">
+        <x:v>Quillajaceae</x:v>
+      </x:c>
+      <x:c r="F7" s="85" t="str">
+        <x:v>Fabales</x:v>
+      </x:c>
+      <x:c r="G7" s="85" t="str">
+        <x:v>aceptado</x:v>
+      </x:c>
+      <x:c r="H7" s="85" t="str">
+        <x:v>urn:lsid:ipni.org:names:731377-1</x:v>
+      </x:c>
+      <x:c r="I7" s="85" t="str">
+        <x:v>Chile Central</x:v>
+      </x:c>
+      <x:c r="J7" s="85" t="str">
+        <x:v>F-020</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="12" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="13" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="30" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="34" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="13" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="13" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="34" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="18" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="20" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="22" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="24" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="42" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="238" t="str">
+        <x:v>Especie ID</x:v>
+      </x:c>
+      <x:c r="B1" s="238" t="str">
+        <x:v>Nombre común</x:v>
+      </x:c>
+      <x:c r="C1" s="238" t="str">
+        <x:v>Rango nativo general</x:v>
+      </x:c>
+      <x:c r="D1" s="238" t="str">
+        <x:v>Regiones Chile registradas</x:v>
+      </x:c>
+      <x:c r="E1" s="238" t="str">
+        <x:v>Altitud min (m)</x:v>
+      </x:c>
+      <x:c r="F1" s="238" t="str">
+        <x:v>Altitud max (m)</x:v>
+      </x:c>
+      <x:c r="G1" s="238" t="str">
+        <x:v>Ecosistema / hábitat registrado</x:v>
+      </x:c>
+      <x:c r="H1" s="238" t="str">
+        <x:v>Hábito foliar</x:v>
+      </x:c>
+      <x:c r="I1" s="238" t="str">
+        <x:v>Floración registrada</x:v>
+      </x:c>
+      <x:c r="J1" s="238" t="str">
+        <x:v>Fuente distribución/altitud</x:v>
+      </x:c>
+      <x:c r="K1" s="238" t="str">
+        <x:v>Fuente ecología/fenología</x:v>
+      </x:c>
+      <x:c r="L1" s="238" t="str">
+        <x:v>Nota</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="85" t="str">
+        <x:v>SP-001</x:v>
+      </x:c>
+      <x:c r="B2" s="85" t="str">
+        <x:v>Peumo</x:v>
+      </x:c>
+      <x:c r="C2" s="85" t="str">
+        <x:v>Chile Central y Chile Sur (POWO)</x:v>
+      </x:c>
+      <x:c r="D2" s="85"/>
+      <x:c r="E2" s="85"/>
+      <x:c r="F2" s="85"/>
+      <x:c r="G2" s="85" t="str">
+        <x:v>bosque esclerófilo</x:v>
+      </x:c>
+      <x:c r="H2" s="85" t="str">
+        <x:v>siempreverde</x:v>
+      </x:c>
+      <x:c r="I2" s="85"/>
+      <x:c r="J2" s="85" t="str">
+        <x:v>F-020</x:v>
+      </x:c>
+      <x:c r="K2" s="85" t="str">
+        <x:v>F-005</x:v>
+      </x:c>
+      <x:c r="L2" s="85" t="str">
+        <x:v>No completar regiones/altitud hasta estructurar una fuente chilena específica ya registrada.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="85" t="str">
+        <x:v>SP-002</x:v>
+      </x:c>
+      <x:c r="B3" s="85" t="str">
+        <x:v>Litre</x:v>
+      </x:c>
+      <x:c r="C3" s="85" t="str">
+        <x:v>Chile Central (POWO)</x:v>
+      </x:c>
+      <x:c r="D3" s="85"/>
+      <x:c r="E3" s="85"/>
+      <x:c r="F3" s="85"/>
+      <x:c r="G3" s="85" t="str">
+        <x:v>formaciones esclerófilas</x:v>
+      </x:c>
+      <x:c r="H3" s="85"/>
+      <x:c r="I3" s="85"/>
+      <x:c r="J3" s="85" t="str">
+        <x:v>F-020</x:v>
+      </x:c>
+      <x:c r="K3" s="85" t="str">
+        <x:v>F-007 / F-008</x:v>
+      </x:c>
+      <x:c r="L3" s="85" t="str">
+        <x:v>La ficha actual no contiene un rango regional/altitudinal estructurado; se conserva como pendiente.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="85" t="str">
+        <x:v>SP-003</x:v>
+      </x:c>
+      <x:c r="B4" s="85" t="str">
+        <x:v>Bollén</x:v>
+      </x:c>
+      <x:c r="C4" s="85" t="str">
+        <x:v>Chile Central (POWO)</x:v>
+      </x:c>
+      <x:c r="D4" s="85"/>
+      <x:c r="E4" s="85"/>
+      <x:c r="F4" s="85"/>
+      <x:c r="G4" s="85"/>
+      <x:c r="H4" s="85"/>
+      <x:c r="I4" s="85"/>
+      <x:c r="J4" s="85" t="str">
+        <x:v>F-020</x:v>
+      </x:c>
+      <x:c r="K4" s="85" t="str">
+        <x:v>F-009</x:v>
+      </x:c>
+      <x:c r="L4" s="85" t="str">
+        <x:v>No inferir rango regional/altitudinal desde la clave morfológica.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="85" t="str">
+        <x:v>SP-004</x:v>
+      </x:c>
+      <x:c r="B5" s="85" t="str">
+        <x:v>Mitique</x:v>
+      </x:c>
+      <x:c r="C5" s="85" t="str">
+        <x:v>Norte-centro y centro de Chile (POWO)</x:v>
+      </x:c>
+      <x:c r="D5" s="85" t="str">
+        <x:v>COQ | VAL | RME | LBO | MAU | NUB</x:v>
+      </x:c>
+      <x:c r="E5" s="85" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F5" s="85" t="n">
+        <x:v>2000</x:v>
+      </x:c>
+      <x:c r="G5" s="85" t="str">
+        <x:v>matorral y bosque esclerófilos</x:v>
+      </x:c>
+      <x:c r="H5" s="85" t="str">
+        <x:v>caducifolio en verano</x:v>
+      </x:c>
+      <x:c r="I5" s="85" t="str">
+        <x:v>primavera</x:v>
+      </x:c>
+      <x:c r="J5" s="85" t="str">
+        <x:v>F-010</x:v>
+      </x:c>
+      <x:c r="K5" s="85" t="str">
+        <x:v>F-011 / F-012</x:v>
+      </x:c>
+      <x:c r="L5" s="85" t="str">
+        <x:v>Caducidad estival es fenológica, no requisito de identificación.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="85" t="str">
+        <x:v>SP-005</x:v>
+      </x:c>
+      <x:c r="B6" s="85" t="str">
+        <x:v>Colliguay</x:v>
+      </x:c>
+      <x:c r="C6" s="85" t="str">
+        <x:v>Norte y centro de Chile (POWO)</x:v>
+      </x:c>
+      <x:c r="D6" s="85" t="str">
+        <x:v>ANT | ATA | COQ | VAL | RME | LBO | MAU | BIO</x:v>
+      </x:c>
+      <x:c r="E6" s="85" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F6" s="85" t="n">
+        <x:v>1300</x:v>
+      </x:c>
+      <x:c r="G6" s="85" t="str">
+        <x:v>matorral mediterráneo; ambientes asoleados y suelos pedregosos</x:v>
+      </x:c>
+      <x:c r="H6" s="85" t="str">
+        <x:v>siempreverde</x:v>
+      </x:c>
+      <x:c r="I6" s="85" t="str">
+        <x:v>mayo–diciembre</x:v>
+      </x:c>
+      <x:c r="J6" s="85" t="str">
+        <x:v>F-013</x:v>
+      </x:c>
+      <x:c r="K6" s="85" t="str">
+        <x:v>F-014 / F-015</x:v>
+      </x:c>
+      <x:c r="L6" s="85"/>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="85" t="str">
+        <x:v>SP-006</x:v>
+      </x:c>
+      <x:c r="B7" s="85" t="str">
+        <x:v>Quillay</x:v>
+      </x:c>
+      <x:c r="C7" s="85" t="str">
+        <x:v>Chile Central (POWO)</x:v>
+      </x:c>
+      <x:c r="D7" s="85" t="str">
+        <x:v>COQ | VAL | RME | LBO | MAU | NUB | BIO | ARA</x:v>
+      </x:c>
+      <x:c r="E7" s="85" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F7" s="85" t="n">
+        <x:v>2000</x:v>
+      </x:c>
+      <x:c r="G7" s="85" t="str">
+        <x:v>formaciones mediterráneas y bosque esclerófilo</x:v>
+      </x:c>
+      <x:c r="H7" s="85" t="str">
+        <x:v>siempreverde</x:v>
+      </x:c>
+      <x:c r="I7" s="85" t="str">
+        <x:v>octubre–enero</x:v>
+      </x:c>
+      <x:c r="J7" s="85" t="str">
+        <x:v>F-016</x:v>
+      </x:c>
+      <x:c r="K7" s="85" t="str">
+        <x:v>F-017 / F-018 / F-019</x:v>
+      </x:c>
+      <x:c r="L7" s="85" t="str">
+        <x:v>Ausencia de flores fuera del periodo no penaliza la identificación.</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="8" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="10" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="30" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="52" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="30" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="20" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="25" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="16" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="10" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="238" t="str">
+        <x:v>Nodo</x:v>
+      </x:c>
+      <x:c r="B1" s="238" t="str">
+        <x:v>Alternativa</x:v>
+      </x:c>
+      <x:c r="C1" s="238" t="str">
+        <x:v>Conjunto candidato antes</x:v>
+      </x:c>
+      <x:c r="D1" s="238" t="str">
+        <x:v>Criterio decisorio</x:v>
+      </x:c>
+      <x:c r="E1" s="238" t="str">
+        <x:v>CAR usados</x:v>
+      </x:c>
+      <x:c r="F1" s="238" t="str">
+        <x:v>Resultado / siguiente</x:v>
+      </x:c>
+      <x:c r="G1" s="238" t="str">
+        <x:v>Rol diagnóstico en piloto</x:v>
+      </x:c>
+      <x:c r="H1" s="238" t="str">
+        <x:v>Seguridad</x:v>
+      </x:c>
+      <x:c r="I1" s="238" t="str">
+        <x:v>Fuente</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="85" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B2" s="85" t="str">
+        <x:v>a</x:v>
+      </x:c>
+      <x:c r="C2" s="85" t="str">
+        <x:v>6 especies</x:v>
+      </x:c>
+      <x:c r="D2" s="85" t="str">
+        <x:v>Hojas opuestas o claramente opuesto-decusadas</x:v>
+      </x:c>
+      <x:c r="E2" s="85" t="str">
+        <x:v>CAR-002 | CAR-025</x:v>
+      </x:c>
+      <x:c r="F2" s="85" t="str">
+        <x:v>Nodo 2</x:v>
+      </x:c>
+      <x:c r="G2" s="85" t="str">
+        <x:v>alto en este conjunto</x:v>
+      </x:c>
+      <x:c r="H2" s="85" t="str">
+        <x:v>seguro</x:v>
+      </x:c>
+      <x:c r="I2" s="85" t="str">
+        <x:v>F-021</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="85" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B3" s="85" t="str">
+        <x:v>b</x:v>
+      </x:c>
+      <x:c r="C3" s="85" t="str">
+        <x:v>6 especies</x:v>
+      </x:c>
+      <x:c r="D3" s="85" t="str">
+        <x:v>Hojas alternas o subopuestas; disposición dudosa no excluye Peumo</x:v>
+      </x:c>
+      <x:c r="E3" s="85" t="str">
+        <x:v>CAR-002</x:v>
+      </x:c>
+      <x:c r="F3" s="85" t="str">
+        <x:v>Nodo 3</x:v>
+      </x:c>
+      <x:c r="G3" s="85" t="str">
+        <x:v>alto, con cautela por Peumo</x:v>
+      </x:c>
+      <x:c r="H3" s="85" t="str">
+        <x:v>seguro</x:v>
+      </x:c>
+      <x:c r="I3" s="85" t="str">
+        <x:v>F-021</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="85" t="str">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B4" s="85" t="str">
+        <x:v>a</x:v>
+      </x:c>
+      <x:c r="C4" s="85" t="str">
+        <x:v>Mitique | Colliguay</x:v>
+      </x:c>
+      <x:c r="D4" s="85" t="str">
+        <x:v>Forma lanceolada/ovado-lanceolada + superficie áspera + patrón decusado</x:v>
+      </x:c>
+      <x:c r="E4" s="85" t="str">
+        <x:v>CAR-008 | CAR-010 | CAR-025</x:v>
+      </x:c>
+      <x:c r="F4" s="85" t="str">
+        <x:v>Mitique</x:v>
+      </x:c>
+      <x:c r="G4" s="85" t="str">
+        <x:v>alto por combinación</x:v>
+      </x:c>
+      <x:c r="H4" s="85" t="str">
+        <x:v>seguro</x:v>
+      </x:c>
+      <x:c r="I4" s="85" t="str">
+        <x:v>F-021</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="85" t="str">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B5" s="85" t="str">
+        <x:v>b</x:v>
+      </x:c>
+      <x:c r="C5" s="85" t="str">
+        <x:v>Mitique | Colliguay</x:v>
+      </x:c>
+      <x:c r="D5" s="85" t="str">
+        <x:v>Hoja oblonga/coriácea + dientes glandulares; cápsula tricoca confirma</x:v>
+      </x:c>
+      <x:c r="E5" s="85" t="str">
+        <x:v>CAR-008 | CAR-004 | CAR-011 | CAR-028</x:v>
+      </x:c>
+      <x:c r="F5" s="85" t="str">
+        <x:v>Colliguay</x:v>
+      </x:c>
+      <x:c r="G5" s="85" t="str">
+        <x:v>alto por combinación</x:v>
+      </x:c>
+      <x:c r="H5" s="85" t="str">
+        <x:v>no cortar</x:v>
+      </x:c>
+      <x:c r="I5" s="85" t="str">
+        <x:v>F-021</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="85" t="str">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B6" s="85" t="str">
+        <x:v>a</x:v>
+      </x:c>
+      <x:c r="C6" s="85" t="str">
+        <x:v>Peumo | Litre | Bollén | Quillay</x:v>
+      </x:c>
+      <x:c r="D6" s="85" t="str">
+        <x:v>Margen aserrado + glándulas en dientes + yema resinosa</x:v>
+      </x:c>
+      <x:c r="E6" s="85" t="str">
+        <x:v>CAR-003 | CAR-011 | CAR-016</x:v>
+      </x:c>
+      <x:c r="F6" s="85" t="str">
+        <x:v>Bollén</x:v>
+      </x:c>
+      <x:c r="G6" s="85" t="str">
+        <x:v>alto por combinación</x:v>
+      </x:c>
+      <x:c r="H6" s="85" t="str">
+        <x:v>seguro</x:v>
+      </x:c>
+      <x:c r="I6" s="85" t="str">
+        <x:v>F-021</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="85" t="str">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B7" s="85" t="str">
+        <x:v>b</x:v>
+      </x:c>
+      <x:c r="C7" s="85" t="str">
+        <x:v>Peumo | Litre | Bollén | Quillay</x:v>
+      </x:c>
+      <x:c r="D7" s="85" t="str">
+        <x:v>No se cumple la combinación diagnóstica de Bollén</x:v>
+      </x:c>
+      <x:c r="E7" s="85" t="str">
+        <x:v>CAR-003 | CAR-011 | CAR-016</x:v>
+      </x:c>
+      <x:c r="F7" s="85" t="str">
+        <x:v>Nodo 4</x:v>
+      </x:c>
+      <x:c r="G7" s="85" t="str">
+        <x:v>filtro de combinación</x:v>
+      </x:c>
+      <x:c r="H7" s="85" t="str">
+        <x:v>seguro</x:v>
+      </x:c>
+      <x:c r="I7" s="85" t="str">
+        <x:v>F-021</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="85" t="str">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B8" s="85" t="str">
+        <x:v>a</x:v>
+      </x:c>
+      <x:c r="C8" s="85" t="str">
+        <x:v>Peumo | Litre | Quillay</x:v>
+      </x:c>
+      <x:c r="D8" s="85" t="str">
+        <x:v>Nervadura clara/amarillenta, nítida y marcadamente prominente</x:v>
+      </x:c>
+      <x:c r="E8" s="85" t="str">
+        <x:v>CAR-022 | CAR-023</x:v>
+      </x:c>
+      <x:c r="F8" s="85" t="str">
+        <x:v>Litre</x:v>
+      </x:c>
+      <x:c r="G8" s="85" t="str">
+        <x:v>alto en este nodo</x:v>
+      </x:c>
+      <x:c r="H8" s="85" t="str">
+        <x:v>precaución</x:v>
+      </x:c>
+      <x:c r="I8" s="85" t="str">
+        <x:v>F-021</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="85" t="str">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B9" s="85" t="str">
+        <x:v>b</x:v>
+      </x:c>
+      <x:c r="C9" s="85" t="str">
+        <x:v>Peumo | Litre | Quillay</x:v>
+      </x:c>
+      <x:c r="D9" s="85" t="str">
+        <x:v>Sin ese patrón de nervadura</x:v>
+      </x:c>
+      <x:c r="E9" s="85" t="str">
+        <x:v>CAR-022 | CAR-023</x:v>
+      </x:c>
+      <x:c r="F9" s="85" t="str">
+        <x:v>Nodo 5</x:v>
+      </x:c>
+      <x:c r="G9" s="85" t="str">
+        <x:v>filtro</x:v>
+      </x:c>
+      <x:c r="H9" s="85" t="str">
+        <x:v>seguro</x:v>
+      </x:c>
+      <x:c r="I9" s="85" t="str">
+        <x:v>F-021</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="85" t="str">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B10" s="85" t="str">
+        <x:v>a</x:v>
+      </x:c>
+      <x:c r="C10" s="85" t="str">
+        <x:v>Peumo | Quillay</x:v>
+      </x:c>
+      <x:c r="D10" s="85" t="str">
+        <x:v>Envés notoriamente más claro, blanquecino a glauco</x:v>
+      </x:c>
+      <x:c r="E10" s="85" t="str">
+        <x:v>CAR-005</x:v>
+      </x:c>
+      <x:c r="F10" s="85" t="str">
+        <x:v>Peumo</x:v>
+      </x:c>
+      <x:c r="G10" s="85" t="str">
+        <x:v>alto en este nodo</x:v>
+      </x:c>
+      <x:c r="H10" s="85" t="str">
+        <x:v>seguro</x:v>
+      </x:c>
+      <x:c r="I10" s="85" t="str">
+        <x:v>F-021</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="85" t="str">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B11" s="85" t="str">
+        <x:v>b</x:v>
+      </x:c>
+      <x:c r="C11" s="85" t="str">
+        <x:v>Peumo | Quillay</x:v>
+      </x:c>
+      <x:c r="D11" s="85" t="str">
+        <x:v>Sin contraste marcado; margen entero a discretamente dentado; frutos confirman</x:v>
+      </x:c>
+      <x:c r="E11" s="85" t="str">
+        <x:v>CAR-003 | CAR-028 | CAR-015</x:v>
+      </x:c>
+      <x:c r="F11" s="85" t="str">
+        <x:v>Quillay</x:v>
+      </x:c>
+      <x:c r="G11" s="85" t="str">
+        <x:v>alto por contexto y confirmación</x:v>
+      </x:c>
+      <x:c r="H11" s="85" t="str">
+        <x:v>seguro</x:v>
+      </x:c>
+      <x:c r="I11" s="85" t="str">
+        <x:v>F-021</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="13" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="28" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="22" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="15" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="22" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="42" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="46" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="40" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="238" t="str">
+        <x:v>ID carácter</x:v>
+      </x:c>
+      <x:c r="B1" s="238" t="str">
+        <x:v>Carácter</x:v>
+      </x:c>
+      <x:c r="C1" s="238" t="str">
+        <x:v>Observación visual directa</x:v>
+      </x:c>
+      <x:c r="D1" s="238" t="str">
+        <x:v>Fotografía</x:v>
+      </x:c>
+      <x:c r="E1" s="238" t="str">
+        <x:v>Interacción necesaria</x:v>
+      </x:c>
+      <x:c r="F1" s="238" t="str">
+        <x:v>Toma / evidencia recomendada</x:v>
+      </x:c>
+      <x:c r="G1" s="238" t="str">
+        <x:v>Restricción de seguridad</x:v>
+      </x:c>
+      <x:c r="H1" s="238" t="str">
+        <x:v>Nota</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="85" t="str">
+        <x:v>CAR-002</x:v>
+      </x:c>
+      <x:c r="B2" s="85" t="str">
+        <x:v>Disposición foliar</x:v>
+      </x:c>
+      <x:c r="C2" s="85" t="str">
+        <x:v>sí</x:v>
+      </x:c>
+      <x:c r="D2" s="85" t="str">
+        <x:v>sí</x:v>
+      </x:c>
+      <x:c r="E2" s="85" t="str">
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="F2" s="85" t="str">
+        <x:v>ramilla con varios nudos</x:v>
+      </x:c>
+      <x:c r="G2" s="85" t="str">
+        <x:v>ninguna</x:v>
+      </x:c>
+      <x:c r="H2" s="85" t="str">
+        <x:v>Una hoja aislada no basta.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="85" t="str">
+        <x:v>CAR-025</x:v>
+      </x:c>
+      <x:c r="B3" s="85" t="str">
+        <x:v>Patrón decusado</x:v>
+      </x:c>
+      <x:c r="C3" s="85" t="str">
+        <x:v>sí</x:v>
+      </x:c>
+      <x:c r="D3" s="85" t="str">
+        <x:v>sí</x:v>
+      </x:c>
+      <x:c r="E3" s="85" t="str">
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="F3" s="85" t="str">
+        <x:v>ramilla con al menos dos pares sucesivos</x:v>
+      </x:c>
+      <x:c r="G3" s="85" t="str">
+        <x:v>ninguna</x:v>
+      </x:c>
+      <x:c r="H3" s="85" t="str">
+        <x:v>Necesita contexto de ramilla.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="85" t="str">
+        <x:v>CAR-003</x:v>
+      </x:c>
+      <x:c r="B4" s="85" t="str">
+        <x:v>Margen foliar</x:v>
+      </x:c>
+      <x:c r="C4" s="85" t="str">
+        <x:v>sí</x:v>
+      </x:c>
+      <x:c r="D4" s="85" t="str">
+        <x:v>sí</x:v>
+      </x:c>
+      <x:c r="E4" s="85" t="str">
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="F4" s="85" t="str">
+        <x:v>hoja completa + acercamiento del borde</x:v>
+      </x:c>
+      <x:c r="G4" s="85" t="str">
+        <x:v>ninguna</x:v>
+      </x:c>
+      <x:c r="H4" s="85" t="str">
+        <x:v>Usar como dentición; ondulación va en CAR-037.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="85" t="str">
+        <x:v>CAR-037</x:v>
+      </x:c>
+      <x:c r="B5" s="85" t="str">
+        <x:v>Ondulación del margen</x:v>
+      </x:c>
+      <x:c r="C5" s="85" t="str">
+        <x:v>sí</x:v>
+      </x:c>
+      <x:c r="D5" s="85" t="str">
+        <x:v>sí</x:v>
+      </x:c>
+      <x:c r="E5" s="85" t="str">
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="F5" s="85" t="str">
+        <x:v>hoja completa en vista plana</x:v>
+      </x:c>
+      <x:c r="G5" s="85" t="str">
+        <x:v>precaución si Litre sigue candidato</x:v>
+      </x:c>
+      <x:c r="H5" s="85" t="str">
+        <x:v>No implica dentición.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="85" t="str">
+        <x:v>CAR-011</x:v>
+      </x:c>
+      <x:c r="B6" s="85" t="str">
+        <x:v>Glándulas en dientes</x:v>
+      </x:c>
+      <x:c r="C6" s="85" t="str">
+        <x:v>sí</x:v>
+      </x:c>
+      <x:c r="D6" s="85" t="str">
+        <x:v>parcial</x:v>
+      </x:c>
+      <x:c r="E6" s="85" t="str">
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="F6" s="85" t="str">
+        <x:v>macro del borde foliar</x:v>
+      </x:c>
+      <x:c r="G6" s="85" t="str">
+        <x:v>ninguna</x:v>
+      </x:c>
+      <x:c r="H6" s="85" t="str">
+        <x:v>Puede requerir buena resolución.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="85" t="str">
+        <x:v>CAR-016</x:v>
+      </x:c>
+      <x:c r="B7" s="85" t="str">
+        <x:v>Yema foliar resinosa</x:v>
+      </x:c>
+      <x:c r="C7" s="85" t="str">
+        <x:v>sí</x:v>
+      </x:c>
+      <x:c r="D7" s="85" t="str">
+        <x:v>parcial</x:v>
+      </x:c>
+      <x:c r="E7" s="85" t="str">
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="F7" s="85" t="str">
+        <x:v>macro de yema/ramilla</x:v>
+      </x:c>
+      <x:c r="G7" s="85" t="str">
+        <x:v>ninguna</x:v>
+      </x:c>
+      <x:c r="H7" s="85" t="str">
+        <x:v>No depender de este carácter si la yema no es visible.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="85" t="str">
+        <x:v>CAR-008</x:v>
+      </x:c>
+      <x:c r="B8" s="85" t="str">
+        <x:v>Forma foliar</x:v>
+      </x:c>
+      <x:c r="C8" s="85" t="str">
+        <x:v>sí</x:v>
+      </x:c>
+      <x:c r="D8" s="85" t="str">
+        <x:v>sí</x:v>
+      </x:c>
+      <x:c r="E8" s="85" t="str">
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="F8" s="85" t="str">
+        <x:v>hoja completa</x:v>
+      </x:c>
+      <x:c r="G8" s="85" t="str">
+        <x:v>ninguna</x:v>
+      </x:c>
+      <x:c r="H8" s="85" t="str">
+        <x:v>Considerar variación intraespecífica.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="85" t="str">
+        <x:v>CAR-010</x:v>
+      </x:c>
+      <x:c r="B9" s="85" t="str">
+        <x:v>Superficie foliar áspera</x:v>
+      </x:c>
+      <x:c r="C9" s="85" t="str">
+        <x:v>sí</x:v>
+      </x:c>
+      <x:c r="D9" s="85" t="str">
+        <x:v>parcial</x:v>
+      </x:c>
+      <x:c r="E9" s="85" t="str">
+        <x:v>no preferente</x:v>
+      </x:c>
+      <x:c r="F9" s="85" t="str">
+        <x:v>luz rasante / detalle de superficie</x:v>
+      </x:c>
+      <x:c r="G9" s="85" t="str">
+        <x:v>no pedir tacto hasta descartar especies de contacto riesgoso</x:v>
+      </x:c>
+      <x:c r="H9" s="85" t="str">
+        <x:v>La fotografía puede no resolver textura.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="85" t="str">
+        <x:v>CAR-022</x:v>
+      </x:c>
+      <x:c r="B10" s="85" t="str">
+        <x:v>Nervio medio prominente</x:v>
+      </x:c>
+      <x:c r="C10" s="85" t="str">
+        <x:v>sí</x:v>
+      </x:c>
+      <x:c r="D10" s="85" t="str">
+        <x:v>sí</x:v>
+      </x:c>
+      <x:c r="E10" s="85" t="str">
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="F10" s="85" t="str">
+        <x:v>hoja con iluminación suficiente</x:v>
+      </x:c>
+      <x:c r="G10" s="85" t="str">
+        <x:v>precaución si Litre sigue candidato</x:v>
+      </x:c>
+      <x:c r="H10" s="85" t="str">
+        <x:v>Combinar con nervaduras secundarias.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="85" t="str">
+        <x:v>CAR-023</x:v>
+      </x:c>
+      <x:c r="B11" s="85" t="str">
+        <x:v>Nervaduras secundarias prominentes</x:v>
+      </x:c>
+      <x:c r="C11" s="85" t="str">
+        <x:v>sí</x:v>
+      </x:c>
+      <x:c r="D11" s="85" t="str">
+        <x:v>sí</x:v>
+      </x:c>
+      <x:c r="E11" s="85" t="str">
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="F11" s="85" t="str">
+        <x:v>detalle de lámina y venación</x:v>
+      </x:c>
+      <x:c r="G11" s="85" t="str">
+        <x:v>precaución si Litre sigue candidato</x:v>
+      </x:c>
+      <x:c r="H11" s="85" t="str">
+        <x:v>Clave para Litre en el nodo 4.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="85" t="str">
+        <x:v>CAR-005</x:v>
+      </x:c>
+      <x:c r="B12" s="85" t="str">
+        <x:v>Coloración del envés</x:v>
+      </x:c>
+      <x:c r="C12" s="85" t="str">
+        <x:v>sí</x:v>
+      </x:c>
+      <x:c r="D12" s="85" t="str">
+        <x:v>sí</x:v>
+      </x:c>
+      <x:c r="E12" s="85" t="str">
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="F12" s="85" t="str">
+        <x:v>fotografía explícita del envés</x:v>
+      </x:c>
+      <x:c r="G12" s="85" t="str">
+        <x:v>precaución si Litre sigue candidato</x:v>
+      </x:c>
+      <x:c r="H12" s="85" t="str">
+        <x:v>La app puede pedir girar la hoja solo si es seguro.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="85" t="str">
+        <x:v>CAR-004</x:v>
+      </x:c>
+      <x:c r="B13" s="85" t="str">
+        <x:v>Consistencia foliar</x:v>
+      </x:c>
+      <x:c r="C13" s="85" t="str">
+        <x:v>sí</x:v>
+      </x:c>
+      <x:c r="D13" s="85" t="str">
+        <x:v>parcial</x:v>
+      </x:c>
+      <x:c r="E13" s="85" t="str">
+        <x:v>no preferente</x:v>
+      </x:c>
+      <x:c r="F13" s="85" t="str">
+        <x:v>foto + contexto; no confiar solo en imagen</x:v>
+      </x:c>
+      <x:c r="G13" s="85" t="str">
+        <x:v>no manipular si Litre sigue candidato</x:v>
+      </x:c>
+      <x:c r="H13" s="85" t="str">
+        <x:v>Rasgo secundario.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="85" t="str">
+        <x:v>CAR-028</x:v>
+      </x:c>
+      <x:c r="B14" s="85" t="str">
+        <x:v>Arquitectura del fruto</x:v>
+      </x:c>
+      <x:c r="C14" s="85" t="str">
+        <x:v>sí</x:v>
+      </x:c>
+      <x:c r="D14" s="85" t="str">
+        <x:v>sí</x:v>
+      </x:c>
+      <x:c r="E14" s="85" t="str">
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="F14" s="85" t="str">
+        <x:v>fruto completo in situ</x:v>
+      </x:c>
+      <x:c r="G14" s="85" t="str">
+        <x:v>no provocar apertura</x:v>
+      </x:c>
+      <x:c r="H14" s="85" t="str">
+        <x:v>Confirmatorio.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="85" t="str">
+        <x:v>CAR-015</x:v>
+      </x:c>
+      <x:c r="B15" s="85" t="str">
+        <x:v>Alas en semillas</x:v>
+      </x:c>
+      <x:c r="C15" s="85" t="str">
+        <x:v>sí</x:v>
+      </x:c>
+      <x:c r="D15" s="85" t="str">
+        <x:v>parcial</x:v>
+      </x:c>
+      <x:c r="E15" s="85" t="str">
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="F15" s="85" t="str">
+        <x:v>semillas visibles naturalmente</x:v>
+      </x:c>
+      <x:c r="G15" s="85" t="str">
+        <x:v>no abrir/cortar fruto para obtenerlas</x:v>
+      </x:c>
+      <x:c r="H15" s="85" t="str">
+        <x:v>Confirmatorio de Quillay.</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="10" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="14" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="30" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="34" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="70" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="70" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="238" t="str">
+        <x:v>Versión</x:v>
+      </x:c>
+      <x:c r="B1" s="238" t="str">
+        <x:v>Fecha</x:v>
+      </x:c>
+      <x:c r="C1" s="238" t="str">
+        <x:v>Alcance</x:v>
+      </x:c>
+      <x:c r="D1" s="238" t="str">
+        <x:v>Estado</x:v>
+      </x:c>
+      <x:c r="E1" s="238" t="str">
+        <x:v>Cambios principales</x:v>
+      </x:c>
+      <x:c r="F1" s="238" t="str">
+        <x:v>Pendientes explícitos</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="85" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="B2" s="85" t="str">
+        <x:v>2026-09-12</x:v>
+      </x:c>
+      <x:c r="C2" s="85" t="str">
+        <x:v>Piloto restringido a SP-001…SP-006</x:v>
+      </x:c>
+      <x:c r="D2" s="85" t="str">
+        <x:v>cierre editorial de base botánica del piloto</x:v>
+      </x:c>
+      <x:c r="E2" s="85" t="str">
+        <x:v>Atomicidad de caracteres; ondulación separada; taxonomía POWO/IPNI; contexto estructurado; poder diagnóstico contextual; observabilidad operativa; clave oficial integrada por referencia.</x:v>
+      </x:c>
+      <x:c r="F2" s="85" t="str">
+        <x:v>Validación empírica de la clave contra las 45 fotos; completar contexto estructurado faltante de Peumo/Litre/Bollén solo con nuevas fuentes/evidencia; no ampliar especies hasta nueva versión.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -12533,11 +14090,33 @@
         <x:v>Estado de ficha</x:v>
       </x:c>
       <x:c r="E8" t="str">
-        <x:v>Ficha avanzada</x:v>
+        <x:v>Ficha botánica v1.0</x:v>
       </x:c>
       <x:c r="F8" t="str"/>
       <x:c r="G8" t="str"/>
       <x:c r="H8" t="str"/>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="245" t="str">
+        <x:v>Autoría taxonómica</x:v>
+      </x:c>
+      <x:c r="B9" s="85" t="str">
+        <x:v>(Molina) Hook. &amp; Arn.</x:v>
+      </x:c>
+      <x:c r="C9" s="85"/>
+      <x:c r="D9" s="245" t="str">
+        <x:v>POWO/IPNI LSID</x:v>
+      </x:c>
+      <x:c r="E9" s="85" t="str">
+        <x:v>urn:lsid:ipni.org:names:69838-1</x:v>
+      </x:c>
+      <x:c r="F9" s="85"/>
+      <x:c r="G9" s="245" t="str">
+        <x:v>Fuente</x:v>
+      </x:c>
+      <x:c r="H9" s="85" t="str">
+        <x:v>F-020</x:v>
+      </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="66" t="str">
@@ -12596,34 +14175,34 @@
       <x:c r="H15" s="66"/>
     </x:row>
     <x:row r="16">
-      <x:c r="A16" s="78" t="str">
+      <x:c r="A16" s="238" t="str">
         <x:v>Carácter</x:v>
       </x:c>
-      <x:c r="B16" s="78" t="str">
+      <x:c r="B16" s="238" t="str">
         <x:v>Estado esperado</x:v>
       </x:c>
-      <x:c r="C16" s="78" t="str">
+      <x:c r="C16" s="238" t="str">
         <x:v>Variabilidad</x:v>
       </x:c>
-      <x:c r="D16" s="78" t="str">
-        <x:v>Detectable en imagen</x:v>
-      </x:c>
-      <x:c r="E16" s="78" t="str">
-        <x:v>Poder diagnóstico</x:v>
-      </x:c>
-      <x:c r="F16" s="78" t="str">
+      <x:c r="D16" s="238" t="str">
+        <x:v>Detectabilidad en imagen (piloto)</x:v>
+      </x:c>
+      <x:c r="E16" s="238" t="str">
+        <x:v>Poder diagnóstico (piloto)</x:v>
+      </x:c>
+      <x:c r="F16" s="238" t="str">
         <x:v>Seguridad</x:v>
       </x:c>
-      <x:c r="G16" s="78" t="str">
-        <x:v>Confianza</x:v>
-      </x:c>
-      <x:c r="H16" s="78" t="str">
+      <x:c r="G16" s="238" t="str">
+        <x:v>Confianza asignación especie–carácter</x:v>
+      </x:c>
+      <x:c r="H16" s="238" t="str">
         <x:v>Fuente</x:v>
       </x:c>
-      <x:c r="I16" s="192" t="str">
+      <x:c r="I16" s="238" t="str">
         <x:v>ID carácter</x:v>
       </x:c>
-      <x:c r="J16" s="192" t="str">
+      <x:c r="J16" s="238" t="str">
         <x:v>Estado normalización</x:v>
       </x:c>
     </x:row>
@@ -12696,7 +14275,7 @@
         <x:v>Margen foliar</x:v>
       </x:c>
       <x:c r="B19" s="94" t="str">
-        <x:v>entero|ondulado</x:v>
+        <x:v>entero</x:v>
       </x:c>
       <x:c r="C19" s="94" t="str">
         <x:v>media</x:v>
@@ -13044,8 +14623,36 @@
       </x:c>
     </x:row>
     <x:row r="30">
-      <x:c r="I30" s="85"/>
-      <x:c r="J30" s="85"/>
+      <x:c r="A30" s="85" t="str">
+        <x:v>Ondulación del margen</x:v>
+      </x:c>
+      <x:c r="B30" s="85" t="str">
+        <x:v>ondulado</x:v>
+      </x:c>
+      <x:c r="C30" s="85" t="str">
+        <x:v>media</x:v>
+      </x:c>
+      <x:c r="D30" s="85" t="str">
+        <x:v>Sí</x:v>
+      </x:c>
+      <x:c r="E30" s="85" t="str">
+        <x:v>medio</x:v>
+      </x:c>
+      <x:c r="F30" s="85" t="str">
+        <x:v>precaucion</x:v>
+      </x:c>
+      <x:c r="G30" s="85" t="str">
+        <x:v>alta</x:v>
+      </x:c>
+      <x:c r="H30" s="85" t="str">
+        <x:v>F-007</x:v>
+      </x:c>
+      <x:c r="I30" s="85" t="str">
+        <x:v>CAR-037</x:v>
+      </x:c>
+      <x:c r="J30" s="85" t="str">
+        <x:v>normalizado</x:v>
+      </x:c>
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="66" t="str">
@@ -13548,11 +15155,33 @@
         <x:v>Estado de ficha</x:v>
       </x:c>
       <x:c r="E8" t="str">
-        <x:v>Ficha avanzada</x:v>
+        <x:v>Ficha botánica v1.0</x:v>
       </x:c>
       <x:c r="F8" t="str"/>
       <x:c r="G8" t="str"/>
       <x:c r="H8" t="str"/>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="245" t="str">
+        <x:v>Autoría taxonómica</x:v>
+      </x:c>
+      <x:c r="B9" s="85" t="str">
+        <x:v>Ruiz &amp; Pav.</x:v>
+      </x:c>
+      <x:c r="C9" s="85"/>
+      <x:c r="D9" s="245" t="str">
+        <x:v>POWO/IPNI LSID</x:v>
+      </x:c>
+      <x:c r="E9" s="85" t="str">
+        <x:v>urn:lsid:ipni.org:names:725811-1</x:v>
+      </x:c>
+      <x:c r="F9" s="85"/>
+      <x:c r="G9" s="245" t="str">
+        <x:v>Fuente</x:v>
+      </x:c>
+      <x:c r="H9" s="85" t="str">
+        <x:v>F-020</x:v>
+      </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="66" t="str">
@@ -13611,34 +15240,34 @@
       <x:c r="H15" s="66"/>
     </x:row>
     <x:row r="16">
-      <x:c r="A16" s="78" t="str">
+      <x:c r="A16" s="238" t="str">
         <x:v>Carácter</x:v>
       </x:c>
-      <x:c r="B16" s="78" t="str">
+      <x:c r="B16" s="238" t="str">
         <x:v>Estado esperado</x:v>
       </x:c>
-      <x:c r="C16" s="78" t="str">
+      <x:c r="C16" s="238" t="str">
         <x:v>Variabilidad</x:v>
       </x:c>
-      <x:c r="D16" s="78" t="str">
-        <x:v>Detectable en imagen</x:v>
-      </x:c>
-      <x:c r="E16" s="78" t="str">
-        <x:v>Poder diagnóstico</x:v>
-      </x:c>
-      <x:c r="F16" s="78" t="str">
+      <x:c r="D16" s="238" t="str">
+        <x:v>Detectabilidad en imagen (piloto)</x:v>
+      </x:c>
+      <x:c r="E16" s="238" t="str">
+        <x:v>Poder diagnóstico (piloto)</x:v>
+      </x:c>
+      <x:c r="F16" s="238" t="str">
         <x:v>Seguridad</x:v>
       </x:c>
-      <x:c r="G16" s="78" t="str">
-        <x:v>Confianza</x:v>
-      </x:c>
-      <x:c r="H16" s="78" t="str">
+      <x:c r="G16" s="238" t="str">
+        <x:v>Confianza asignación especie–carácter</x:v>
+      </x:c>
+      <x:c r="H16" s="238" t="str">
         <x:v>Fuente</x:v>
       </x:c>
-      <x:c r="I16" s="192" t="str">
+      <x:c r="I16" s="238" t="str">
         <x:v>ID carácter</x:v>
       </x:c>
-      <x:c r="J16" s="192" t="str">
+      <x:c r="J16" s="238" t="str">
         <x:v>Estado normalización</x:v>
       </x:c>
     </x:row>
@@ -14439,11 +16068,33 @@
         <x:v>Estado de ficha</x:v>
       </x:c>
       <x:c r="E8" t="str">
-        <x:v>Ficha avanzada</x:v>
+        <x:v>Ficha botánica v1.0</x:v>
       </x:c>
       <x:c r="F8" t="str"/>
       <x:c r="G8" t="str"/>
       <x:c r="H8" t="str"/>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="245" t="str">
+        <x:v>Autoría taxonómica</x:v>
+      </x:c>
+      <x:c r="B9" s="85" t="str">
+        <x:v>Lindl.</x:v>
+      </x:c>
+      <x:c r="C9" s="85"/>
+      <x:c r="D9" s="245" t="str">
+        <x:v>POWO/IPNI LSID</x:v>
+      </x:c>
+      <x:c r="E9" s="85" t="str">
+        <x:v>urn:lsid:ipni.org:names:238927-1</x:v>
+      </x:c>
+      <x:c r="F9" s="85"/>
+      <x:c r="G9" s="245" t="str">
+        <x:v>Fuente</x:v>
+      </x:c>
+      <x:c r="H9" s="85" t="str">
+        <x:v>F-020</x:v>
+      </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="66" t="str">
@@ -14502,34 +16153,34 @@
       <x:c r="H15" s="66"/>
     </x:row>
     <x:row r="16">
-      <x:c r="A16" s="125" t="str">
+      <x:c r="A16" s="238" t="str">
         <x:v>Carácter</x:v>
       </x:c>
-      <x:c r="B16" s="125" t="str">
+      <x:c r="B16" s="238" t="str">
         <x:v>Estado esperado</x:v>
       </x:c>
-      <x:c r="C16" s="125" t="str">
+      <x:c r="C16" s="238" t="str">
         <x:v>Variabilidad</x:v>
       </x:c>
-      <x:c r="D16" s="125" t="str">
-        <x:v>Detectable en imagen</x:v>
-      </x:c>
-      <x:c r="E16" s="125" t="str">
-        <x:v>Poder diagnóstico</x:v>
-      </x:c>
-      <x:c r="F16" s="125" t="str">
+      <x:c r="D16" s="238" t="str">
+        <x:v>Detectabilidad en imagen (piloto)</x:v>
+      </x:c>
+      <x:c r="E16" s="238" t="str">
+        <x:v>Poder diagnóstico (piloto)</x:v>
+      </x:c>
+      <x:c r="F16" s="238" t="str">
         <x:v>Seguridad</x:v>
       </x:c>
-      <x:c r="G16" s="125" t="str">
-        <x:v>Confianza</x:v>
-      </x:c>
-      <x:c r="H16" s="125" t="str">
+      <x:c r="G16" s="238" t="str">
+        <x:v>Confianza asignación especie–carácter</x:v>
+      </x:c>
+      <x:c r="H16" s="238" t="str">
         <x:v>Fuente</x:v>
       </x:c>
-      <x:c r="I16" s="192" t="str">
+      <x:c r="I16" s="238" t="str">
         <x:v>ID carácter</x:v>
       </x:c>
-      <x:c r="J16" s="192" t="str">
+      <x:c r="J16" s="238" t="str">
         <x:v>Estado normalización</x:v>
       </x:c>
     </x:row>
@@ -15267,11 +16918,33 @@
         <x:v>Estado de ficha</x:v>
       </x:c>
       <x:c r="E8" t="str">
-        <x:v>Ficha avanzada</x:v>
+        <x:v>Ficha botánica v1.0</x:v>
       </x:c>
       <x:c r="F8" t="str"/>
       <x:c r="G8" t="str"/>
       <x:c r="H8" t="str"/>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="245" t="str">
+        <x:v>Autoría taxonómica</x:v>
+      </x:c>
+      <x:c r="B9" s="85" t="str">
+        <x:v>Molina</x:v>
+      </x:c>
+      <x:c r="C9" s="85"/>
+      <x:c r="D9" s="245" t="str">
+        <x:v>POWO/IPNI LSID</x:v>
+      </x:c>
+      <x:c r="E9" s="85" t="str">
+        <x:v>urn:lsid:ipni.org:names:341899-1</x:v>
+      </x:c>
+      <x:c r="F9" s="85"/>
+      <x:c r="G9" s="245" t="str">
+        <x:v>Fuente</x:v>
+      </x:c>
+      <x:c r="H9" s="85" t="str">
+        <x:v>F-020</x:v>
+      </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="66" t="str">
@@ -15330,34 +17003,34 @@
       <x:c r="H15" s="66"/>
     </x:row>
     <x:row r="16">
-      <x:c r="A16" s="141" t="str">
+      <x:c r="A16" s="238" t="str">
         <x:v>Carácter</x:v>
       </x:c>
-      <x:c r="B16" s="141" t="str">
+      <x:c r="B16" s="238" t="str">
         <x:v>Estado esperado</x:v>
       </x:c>
-      <x:c r="C16" s="141" t="str">
+      <x:c r="C16" s="238" t="str">
         <x:v>Variabilidad</x:v>
       </x:c>
-      <x:c r="D16" s="141" t="str">
-        <x:v>Detectable en imagen</x:v>
-      </x:c>
-      <x:c r="E16" s="141" t="str">
-        <x:v>Poder diagnóstico</x:v>
-      </x:c>
-      <x:c r="F16" s="141" t="str">
+      <x:c r="D16" s="238" t="str">
+        <x:v>Detectabilidad en imagen (piloto)</x:v>
+      </x:c>
+      <x:c r="E16" s="238" t="str">
+        <x:v>Poder diagnóstico (piloto)</x:v>
+      </x:c>
+      <x:c r="F16" s="238" t="str">
         <x:v>Seguridad</x:v>
       </x:c>
-      <x:c r="G16" s="141" t="str">
-        <x:v>Confianza</x:v>
-      </x:c>
-      <x:c r="H16" s="141" t="str">
+      <x:c r="G16" s="238" t="str">
+        <x:v>Confianza asignación especie–carácter</x:v>
+      </x:c>
+      <x:c r="H16" s="238" t="str">
         <x:v>Fuente</x:v>
       </x:c>
-      <x:c r="I16" s="192" t="str">
+      <x:c r="I16" s="238" t="str">
         <x:v>ID carácter</x:v>
       </x:c>
-      <x:c r="J16" s="192" t="str">
+      <x:c r="J16" s="238" t="str">
         <x:v>Estado normalización</x:v>
       </x:c>
     </x:row>
@@ -16062,11 +17735,33 @@
         <x:v>Estado de ficha</x:v>
       </x:c>
       <x:c r="E8" t="str">
-        <x:v>Ficha avanzada</x:v>
+        <x:v>Ficha botánica v1.0</x:v>
       </x:c>
       <x:c r="F8" t="str"/>
       <x:c r="G8" t="str"/>
       <x:c r="H8" t="str"/>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="245" t="str">
+        <x:v>Autoría taxonómica</x:v>
+      </x:c>
+      <x:c r="B9" s="85" t="str">
+        <x:v>Molina</x:v>
+      </x:c>
+      <x:c r="C9" s="85"/>
+      <x:c r="D9" s="245" t="str">
+        <x:v>POWO/IPNI LSID</x:v>
+      </x:c>
+      <x:c r="E9" s="85" t="str">
+        <x:v>urn:lsid:ipni.org:names:731377-1</x:v>
+      </x:c>
+      <x:c r="F9" s="85"/>
+      <x:c r="G9" s="245" t="str">
+        <x:v>Fuente</x:v>
+      </x:c>
+      <x:c r="H9" s="85" t="str">
+        <x:v>F-020</x:v>
+      </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="66" t="str">
@@ -16125,34 +17820,34 @@
       <x:c r="H15" s="66"/>
     </x:row>
     <x:row r="16">
-      <x:c r="A16" s="151" t="str">
+      <x:c r="A16" s="238" t="str">
         <x:v>Carácter</x:v>
       </x:c>
-      <x:c r="B16" s="151" t="str">
+      <x:c r="B16" s="238" t="str">
         <x:v>Estado esperado</x:v>
       </x:c>
-      <x:c r="C16" s="151" t="str">
+      <x:c r="C16" s="238" t="str">
         <x:v>Variabilidad</x:v>
       </x:c>
-      <x:c r="D16" s="151" t="str">
-        <x:v>Detectable en imagen</x:v>
-      </x:c>
-      <x:c r="E16" s="151" t="str">
-        <x:v>Poder diagnóstico</x:v>
-      </x:c>
-      <x:c r="F16" s="151" t="str">
+      <x:c r="D16" s="238" t="str">
+        <x:v>Detectabilidad en imagen (piloto)</x:v>
+      </x:c>
+      <x:c r="E16" s="238" t="str">
+        <x:v>Poder diagnóstico (piloto)</x:v>
+      </x:c>
+      <x:c r="F16" s="238" t="str">
         <x:v>Seguridad</x:v>
       </x:c>
-      <x:c r="G16" s="151" t="str">
-        <x:v>Confianza</x:v>
-      </x:c>
-      <x:c r="H16" s="151" t="str">
+      <x:c r="G16" s="238" t="str">
+        <x:v>Confianza asignación especie–carácter</x:v>
+      </x:c>
+      <x:c r="H16" s="238" t="str">
         <x:v>Fuente</x:v>
       </x:c>
-      <x:c r="I16" s="192" t="str">
+      <x:c r="I16" s="238" t="str">
         <x:v>ID carácter</x:v>
       </x:c>
-      <x:c r="J16" s="192" t="str">
+      <x:c r="J16" s="238" t="str">
         <x:v>Estado normalización</x:v>
       </x:c>
     </x:row>
@@ -16743,22 +18438,22 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="77" t="str">
+      <x:c r="A1" s="238" t="str">
         <x:v>Fuente ID</x:v>
       </x:c>
-      <x:c r="B1" s="77" t="str">
+      <x:c r="B1" s="238" t="str">
         <x:v>Tipo</x:v>
       </x:c>
-      <x:c r="C1" s="77" t="str">
+      <x:c r="C1" s="238" t="str">
         <x:v>Referencia</x:v>
       </x:c>
-      <x:c r="D1" s="77" t="str">
+      <x:c r="D1" s="238" t="str">
         <x:v>Uso prioritario</x:v>
       </x:c>
-      <x:c r="E1" s="77" t="str">
+      <x:c r="E1" s="238" t="str">
         <x:v>URL</x:v>
       </x:c>
-      <x:c r="F1" s="77" t="str">
+      <x:c r="F1" s="238" t="str">
         <x:v>Notas</x:v>
       </x:c>
     </x:row>
@@ -17136,6 +18831,46 @@
       </x:c>
       <x:c r="F20" s="85" t="str">
         <x:v>Árbol siempreverde; hojas simples alternas duras; flores estrelladas blanco-amarillentas; fruto de cinco secciones con semillas aladas; floración octubre-enero.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" t="str">
+        <x:v>F-020</x:v>
+      </x:c>
+      <x:c r="B21" t="str">
+        <x:v>Base taxonómica internacional</x:v>
+      </x:c>
+      <x:c r="C21" t="str">
+        <x:v>Royal Botanic Gardens, Kew. Plants of the World Online (POWO) / IPNI backbone.</x:v>
+      </x:c>
+      <x:c r="D21" t="str">
+        <x:v>Autoría, nombre aceptado, estado taxonómico, clasificación y rango nativo general</x:v>
+      </x:c>
+      <x:c r="E21" t="str">
+        <x:v>https://powo.science.kew.org/</x:v>
+      </x:c>
+      <x:c r="F21" t="str">
+        <x:v>Consulta 2026-09-12. Los LSID específicos se registran en la hoja Taxonomia.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" t="str">
+        <x:v>F-021</x:v>
+      </x:c>
+      <x:c r="B22" t="str">
+        <x:v>Documento interno / clave</x:v>
+      </x:c>
+      <x:c r="C22" t="str">
+        <x:v>Árboris. Clave botánica del piloto, versión 1.0 revisada.</x:v>
+      </x:c>
+      <x:c r="D22" t="str">
+        <x:v>Orden de preguntas, contexto discriminativo y seguridad del piloto de seis especies</x:v>
+      </x:c>
+      <x:c r="E22" t="str">
+        <x:v>https://drive.google.com/file/d/1tvgWaLW0DwuZO2b4z3i9e5vBulUkM0xy</x:v>
+      </x:c>
+      <x:c r="F22" t="str">
+        <x:v>Derivada de las fuentes botánicas del piloto; no reemplaza las fuentes primarias.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -18781,7 +20516,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R405f685e564a461c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R98af92b8618847cf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>